<commit_message>
Update to US October CMA
</commit_message>
<xml_diff>
--- a/US/October CMA/US October CMA Data.xlsx
+++ b/US/October CMA/US October CMA Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coledushin/Documents/GWHS/US/October CMA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E05B8F56-15BC-3B46-AEF1-F2FAB66D4ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD1D701F-00E1-FC40-BFA0-DB41C9C233F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="15520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scores" sheetId="1" r:id="rId1"/>
@@ -2586,12 +2586,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF356854"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2696,7 +2698,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2790,7 +2792,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
@@ -2801,27 +2802,6 @@
     <cellStyle name="Percent 2" xfId="4" xr:uid="{E6DE421D-B06A-DB4D-BCE7-D696BB42B3F4}"/>
   </cellStyles>
   <dxfs count="32">
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2844,6 +2824,12 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF1F3A2E"/>
       </font>
@@ -2853,7 +2839,37 @@
       <font>
         <color rgb="FF1F3A2E"/>
       </font>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
       <font>
@@ -2878,6 +2894,97 @@
         <color rgb="FF1F3A2E"/>
       </font>
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F3A2E"/>
+      </font>
+      <alignment vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF1F3A2E"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -2937,119 +3044,13 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF1F3A2E"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F3A2E"/>
-      </font>
-      <alignment vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Light and Airy" count="4" xr9:uid="{9857ACD9-B079-C44A-A030-69F7726DB419}">
-      <tableStyleElement type="wholeTable" dxfId="15"/>
-      <tableStyleElement type="headerRow" dxfId="14"/>
-      <tableStyleElement type="totalRow" dxfId="13"/>
-      <tableStyleElement type="firstRowStripe" dxfId="12"/>
+      <tableStyleElement type="wholeTable" dxfId="31"/>
+      <tableStyleElement type="headerRow" dxfId="30"/>
+      <tableStyleElement type="totalRow" dxfId="29"/>
+      <tableStyleElement type="firstRowStripe" dxfId="28"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -3091,7 +3092,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Scores" displayName="Scores" ref="A1:V94" totalsRowCount="1" headerRowDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Scores" displayName="Scores" ref="A1:V94" totalsRowCount="1" headerRowDxfId="26">
   <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Student"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="First"/>
@@ -3099,8 +3100,8 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Class"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Period"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC" totalsRowFunction="average" totalsRowDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC" totalsRowFunction="average" totalsRowDxfId="24"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Final"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="2"/>
@@ -3121,25 +3122,25 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="20" dataDxfId="18" totalsRowDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="23" dataDxfId="22" totalsRowDxfId="21">
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="25"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="24"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="23"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="22"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3149,7 +3150,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:B19">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Model"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3160,7 +3161,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Standard"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Concept"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3172,7 +3173,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="#"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Framework"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Specifications"/>
-    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.CONCAT(Table3[[#This Row],['#]],": ",Table3[[#This Row],[Framework]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3408,9 +3409,8 @@
   <cols>
     <col min="1" max="3" width="22.6640625" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="15" width="10.1640625" customWidth="1"/>
-    <col min="16" max="16" width="10.1640625" customWidth="1" collapsed="1"/>
-    <col min="17" max="22" width="10.1640625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="16" width="10.1640625" customWidth="1"/>
+    <col min="17" max="22" width="10.1640625" customWidth="1" outlineLevel="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="16" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -10161,7 +10161,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:O93">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>Q2=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10189,10 +10189,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="10.1640625" customWidth="1"/>
-    <col min="3" max="3" width="37.6640625" customWidth="1"/>
-    <col min="4" max="4" width="37.6640625" style="29" customWidth="1"/>
+    <col min="3" max="4" width="37.6640625" customWidth="1"/>
     <col min="5" max="5" width="10.1640625" customWidth="1"/>
-    <col min="6" max="9" width="25.1640625" style="29" customWidth="1"/>
+    <col min="6" max="9" width="25.1640625" customWidth="1"/>
     <col min="10" max="10" width="19.1640625" customWidth="1"/>
     <col min="11" max="11" width="17.83203125" customWidth="1"/>
     <col min="12" max="12" width="17.6640625" customWidth="1"/>
@@ -10601,7 +10600,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:I8">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>"Option_"&amp;$E2=F$1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11327,7 +11326,7 @@
       <c r="C1" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="29" t="s">
         <v>840</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Bermejo US Oct SEQ scores
</commit_message>
<xml_diff>
--- a/US/October CMA/US October CMA Data.xlsx
+++ b/US/October CMA/US October CMA Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coledushin/Documents/GWHS/US/October CMA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDF4E09-BA8B-6A46-A101-51047F14F5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA37C0E-5382-C047-830C-CED48E380BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3362,114 +3362,6 @@
   </cellStyles>
   <dxfs count="76">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF3F4A58"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FF3F4A58"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF3F4A58"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF3F4A58"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF3F4A58"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF3F4A58"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3534,6 +3426,60 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF3F4A58"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF3F4A58"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF3F4A58"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF3F4A58"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3549,102 +3495,25 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF3F4A58"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF3F4A58"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color rgb="FF3F4A58"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
+        <color rgb="FF9C0006"/>
       </font>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -3786,6 +3655,137 @@
       <alignment vertical="center"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF3F4A58"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF3F4A58"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FF3F4A58"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF3F4A58"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF3F4A58"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFF5F8FB"/>
@@ -3892,57 +3892,57 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Scores" displayName="Scores" ref="A1:V121" totalsRowCount="1" headerRowDxfId="48" dataDxfId="47" totalsRowDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Scores" displayName="Scores" ref="A1:V121" totalsRowCount="1" headerRowDxfId="71" dataDxfId="70" totalsRowDxfId="69">
   <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Student" dataDxfId="45" totalsRowDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="First" dataDxfId="44" totalsRowDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Last" dataDxfId="43" totalsRowDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Class" dataDxfId="42" totalsRowDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Period" dataDxfId="41" totalsRowDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL" dataDxfId="5" totalsRowDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="4" totalsRowDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC" totalsRowFunction="custom" dataDxfId="40" totalsRowDxfId="20">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Student" dataDxfId="68" totalsRowDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="First" dataDxfId="67" totalsRowDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Last" dataDxfId="66" totalsRowDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Class" dataDxfId="65" totalsRowDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Period" dataDxfId="64" totalsRowDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL" dataDxfId="63" totalsRowDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="62" totalsRowDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="14">
       <totalsRowFormula>AVERAGE(Scores[MC])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Final" dataDxfId="39" totalsRowDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1" dataDxfId="38" totalsRowDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="2" dataDxfId="37" totalsRowDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="3" dataDxfId="36" totalsRowDxfId="16"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="4" dataDxfId="35" totalsRowDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="5" dataDxfId="34" totalsRowDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="6" dataDxfId="33" totalsRowDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="SEQ" dataDxfId="32" totalsRowDxfId="12"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Q1" dataDxfId="31" totalsRowDxfId="11"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Q2" dataDxfId="30" totalsRowDxfId="10"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Q3" dataDxfId="29" totalsRowDxfId="9"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Q4" dataDxfId="28" totalsRowDxfId="8"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Q5" dataDxfId="27" totalsRowDxfId="7"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Q6" dataDxfId="26" totalsRowDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Final" dataDxfId="60" totalsRowDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1" dataDxfId="59" totalsRowDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="2" dataDxfId="58" totalsRowDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="3" dataDxfId="57" totalsRowDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="4" dataDxfId="56" totalsRowDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="5" dataDxfId="55" totalsRowDxfId="8"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="6" dataDxfId="54" totalsRowDxfId="7"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="SEQ" dataDxfId="53" totalsRowDxfId="6"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Q1" dataDxfId="52" totalsRowDxfId="5"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Q2" dataDxfId="51" totalsRowDxfId="4"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Q3" dataDxfId="50" totalsRowDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Q4" dataDxfId="49" totalsRowDxfId="2"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Q5" dataDxfId="48" totalsRowDxfId="1"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Q6" dataDxfId="47" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="71" dataDxfId="70" totalsRowDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="46" dataDxfId="45" totalsRowDxfId="44">
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="66"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="64"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="62"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="61"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="60"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="59"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="58"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="57"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="56"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="55"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="54"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="53"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="35"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="34"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="33"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="32"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="31"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="30"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="29"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="28"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3952,7 +3952,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:B19">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Model"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3963,7 +3963,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Standard"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Concept"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3975,7 +3975,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="#"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Framework"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Specifications"/>
-    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="49">
+    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="24">
       <calculatedColumnFormula>_xlfn.CONCAT(Table3[[#This Row],['#]],": ",Table3[[#This Row],[Framework]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4337,7 +4337,9 @@
       <c r="O2" s="1">
         <v>2</v>
       </c>
-      <c r="P2" s="28"/>
+      <c r="P2" s="28">
+        <v>3</v>
+      </c>
       <c r="Q2" s="1">
         <f>IF(J2=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4413,7 +4415,9 @@
       <c r="O3" s="1">
         <v>3</v>
       </c>
-      <c r="P3" s="28"/>
+      <c r="P3" s="28">
+        <v>1</v>
+      </c>
       <c r="Q3" s="1">
         <f>IF(J3=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4489,7 +4493,9 @@
       <c r="O4" s="1">
         <v>1</v>
       </c>
-      <c r="P4" s="28"/>
+      <c r="P4" s="28">
+        <v>2</v>
+      </c>
       <c r="Q4" s="1">
         <f>IF(J4=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4565,7 +4571,9 @@
       <c r="O5" s="1">
         <v>2</v>
       </c>
-      <c r="P5" s="28"/>
+      <c r="P5" s="28">
+        <v>1</v>
+      </c>
       <c r="Q5" s="1">
         <f>IF(J5=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4641,7 +4649,9 @@
       <c r="O6" s="1">
         <v>2</v>
       </c>
-      <c r="P6" s="28"/>
+      <c r="P6" s="28">
+        <v>1</v>
+      </c>
       <c r="Q6" s="1">
         <f>IF(J6=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4717,7 +4727,9 @@
       <c r="O7" s="1">
         <v>3</v>
       </c>
-      <c r="P7" s="28"/>
+      <c r="P7" s="28">
+        <v>1</v>
+      </c>
       <c r="Q7" s="1">
         <f>IF(J7=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4793,7 +4805,9 @@
       <c r="O8" s="1">
         <v>2</v>
       </c>
-      <c r="P8" s="28"/>
+      <c r="P8" s="28">
+        <v>1</v>
+      </c>
       <c r="Q8" s="1">
         <f>IF(J8=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -4869,7 +4883,9 @@
       <c r="O9" s="1">
         <v>2</v>
       </c>
-      <c r="P9" s="28"/>
+      <c r="P9" s="28">
+        <v>1</v>
+      </c>
       <c r="Q9" s="1">
         <f>IF(J9=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -4945,7 +4961,9 @@
       <c r="O10" s="1">
         <v>2</v>
       </c>
-      <c r="P10" s="28"/>
+      <c r="P10" s="28">
+        <v>0</v>
+      </c>
       <c r="Q10" s="1">
         <f>IF(J10=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5019,7 +5037,9 @@
       <c r="O11" s="1">
         <v>3</v>
       </c>
-      <c r="P11" s="28"/>
+      <c r="P11" s="28">
+        <v>3</v>
+      </c>
       <c r="Q11" s="1">
         <f>IF(J11=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5095,7 +5115,9 @@
       <c r="O12" s="1">
         <v>1</v>
       </c>
-      <c r="P12" s="28"/>
+      <c r="P12" s="28">
+        <v>1</v>
+      </c>
       <c r="Q12" s="1">
         <f>IF(J12=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5171,7 +5193,9 @@
       <c r="O13" s="1">
         <v>2</v>
       </c>
-      <c r="P13" s="28"/>
+      <c r="P13" s="28">
+        <v>3</v>
+      </c>
       <c r="Q13" s="1">
         <f>IF(J13=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -5247,7 +5271,9 @@
       <c r="O14" s="1">
         <v>1</v>
       </c>
-      <c r="P14" s="28"/>
+      <c r="P14" s="28">
+        <v>0</v>
+      </c>
       <c r="Q14" s="1">
         <f>IF(J14=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5323,7 +5349,9 @@
       <c r="O15" s="1">
         <v>4</v>
       </c>
-      <c r="P15" s="28"/>
+      <c r="P15" s="28">
+        <v>1</v>
+      </c>
       <c r="Q15" s="1">
         <f>IF(J15=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5399,7 +5427,9 @@
       <c r="O16" s="1">
         <v>2</v>
       </c>
-      <c r="P16" s="28"/>
+      <c r="P16" s="28">
+        <v>2</v>
+      </c>
       <c r="Q16" s="1">
         <f>IF(J16=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -5475,7 +5505,9 @@
       <c r="O17" s="1">
         <v>2</v>
       </c>
-      <c r="P17" s="28"/>
+      <c r="P17" s="28">
+        <v>2</v>
+      </c>
       <c r="Q17" s="1">
         <f>IF(J17=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -5551,7 +5583,9 @@
       <c r="O18" s="1">
         <v>4</v>
       </c>
-      <c r="P18" s="28"/>
+      <c r="P18" s="28">
+        <v>3</v>
+      </c>
       <c r="Q18" s="1">
         <f>IF(J18=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5627,7 +5661,9 @@
       <c r="O19" s="1">
         <v>2</v>
       </c>
-      <c r="P19" s="28"/>
+      <c r="P19" s="28">
+        <v>1</v>
+      </c>
       <c r="Q19" s="1">
         <f>IF(J19=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5841,7 +5877,9 @@
       <c r="O22" s="1">
         <v>2</v>
       </c>
-      <c r="P22" s="28"/>
+      <c r="P22" s="28">
+        <v>2</v>
+      </c>
       <c r="Q22" s="1">
         <f>IF(J22=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5917,7 +5955,9 @@
       <c r="O23" s="1">
         <v>2</v>
       </c>
-      <c r="P23" s="28"/>
+      <c r="P23" s="28">
+        <v>1</v>
+      </c>
       <c r="Q23" s="1">
         <f>IF(J23=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -5993,7 +6033,9 @@
       <c r="O24" s="1">
         <v>2</v>
       </c>
-      <c r="P24" s="28"/>
+      <c r="P24" s="28">
+        <v>1</v>
+      </c>
       <c r="Q24" s="1">
         <f>IF(J24=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -6069,7 +6111,9 @@
       <c r="O25" s="1">
         <v>4</v>
       </c>
-      <c r="P25" s="28"/>
+      <c r="P25" s="28">
+        <v>1</v>
+      </c>
       <c r="Q25" s="1">
         <f>IF(J25=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -6145,7 +6189,9 @@
       <c r="O26" s="1">
         <v>4</v>
       </c>
-      <c r="P26" s="28"/>
+      <c r="P26" s="28">
+        <v>1</v>
+      </c>
       <c r="Q26" s="1">
         <f>IF(J26=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -6221,7 +6267,9 @@
       <c r="O27" s="1">
         <v>1</v>
       </c>
-      <c r="P27" s="28"/>
+      <c r="P27" s="28">
+        <v>2</v>
+      </c>
       <c r="Q27" s="1">
         <f>IF(J27=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -6297,7 +6345,9 @@
       <c r="O28" s="1">
         <v>2</v>
       </c>
-      <c r="P28" s="28"/>
+      <c r="P28" s="28">
+        <v>3</v>
+      </c>
       <c r="Q28" s="1">
         <f>IF(J28=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -8057,7 +8107,9 @@
       <c r="O52" s="1">
         <v>2</v>
       </c>
-      <c r="P52" s="28"/>
+      <c r="P52" s="28">
+        <v>3</v>
+      </c>
       <c r="Q52" s="1">
         <v>0</v>
       </c>
@@ -8124,7 +8176,9 @@
       <c r="O53" s="1">
         <v>2</v>
       </c>
-      <c r="P53" s="28"/>
+      <c r="P53" s="28">
+        <v>1</v>
+      </c>
       <c r="Q53" s="1">
         <v>0</v>
       </c>
@@ -8258,7 +8312,9 @@
       <c r="O55" s="1">
         <v>2</v>
       </c>
-      <c r="P55" s="28"/>
+      <c r="P55" s="28">
+        <v>3</v>
+      </c>
       <c r="Q55" s="1">
         <v>1</v>
       </c>
@@ -8392,7 +8448,9 @@
       <c r="O57" s="1">
         <v>2</v>
       </c>
-      <c r="P57" s="28"/>
+      <c r="P57" s="28">
+        <v>4</v>
+      </c>
       <c r="Q57" s="1">
         <v>1</v>
       </c>
@@ -8459,7 +8517,9 @@
       <c r="O58" s="1">
         <v>2</v>
       </c>
-      <c r="P58" s="28"/>
+      <c r="P58" s="28">
+        <v>4</v>
+      </c>
       <c r="Q58" s="1">
         <v>1</v>
       </c>
@@ -8526,7 +8586,9 @@
       <c r="O59" s="1">
         <v>2</v>
       </c>
-      <c r="P59" s="28"/>
+      <c r="P59" s="28">
+        <v>4</v>
+      </c>
       <c r="Q59" s="1">
         <v>1</v>
       </c>
@@ -8656,7 +8718,9 @@
       <c r="O61" s="1">
         <v>2</v>
       </c>
-      <c r="P61" s="28"/>
+      <c r="P61" s="28">
+        <v>4</v>
+      </c>
       <c r="Q61" s="1">
         <v>0</v>
       </c>
@@ -8857,7 +8921,9 @@
       <c r="O64" s="1">
         <v>2</v>
       </c>
-      <c r="P64" s="28"/>
+      <c r="P64" s="28">
+        <v>4</v>
+      </c>
       <c r="Q64" s="1">
         <v>1</v>
       </c>
@@ -9058,7 +9124,9 @@
       <c r="O67" s="1">
         <v>2</v>
       </c>
-      <c r="P67" s="28"/>
+      <c r="P67" s="28">
+        <v>4</v>
+      </c>
       <c r="Q67" s="1">
         <v>1</v>
       </c>
@@ -9125,7 +9193,9 @@
       <c r="O68" s="1">
         <v>2</v>
       </c>
-      <c r="P68" s="28"/>
+      <c r="P68" s="28">
+        <v>3</v>
+      </c>
       <c r="Q68" s="1">
         <v>1</v>
       </c>
@@ -12634,7 +12704,7 @@
   </sheetData>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="J2:O120">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>Q2=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13073,7 +13143,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:I8">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="22" priority="1">
       <formula>"Option_"&amp;$E2=F$1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Added Dushin Oct SEQ
</commit_message>
<xml_diff>
--- a/US/October CMA/US October CMA Data.xlsx
+++ b/US/October CMA/US October CMA Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coledushin/Documents/GWHS/US/October CMA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BCB3DD-D386-CB45-9D79-6E9E13CF17BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{146F52D6-DE9F-D44A-89FE-326FE8B2944C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3501,9 +3501,6 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF006100"/>
       </font>
@@ -3763,6 +3760,9 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3908,51 +3908,51 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Last" dataDxfId="68" totalsRowDxfId="20"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Class" dataDxfId="67" totalsRowDxfId="19"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Period" dataDxfId="66" totalsRowDxfId="18"/>
-    <tableColumn id="24" xr3:uid="{3D78B174-0EEB-C04D-AFAA-846CD92209B4}" name="Grade" dataDxfId="23" totalsRowDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL" dataDxfId="65" totalsRowDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="64" totalsRowDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="14">
+    <tableColumn id="24" xr3:uid="{3D78B174-0EEB-C04D-AFAA-846CD92209B4}" name="Grade" dataDxfId="65" totalsRowDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ELL" dataDxfId="64" totalsRowDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="IEP" dataDxfId="63" totalsRowDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MC" totalsRowFunction="custom" dataDxfId="62" totalsRowDxfId="14">
       <totalsRowFormula>AVERAGE(Scores[MC])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Final" dataDxfId="62" totalsRowDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1" dataDxfId="61" totalsRowDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="2" dataDxfId="60" totalsRowDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="3" dataDxfId="59" totalsRowDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="4" dataDxfId="58" totalsRowDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="5" dataDxfId="57" totalsRowDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="6" dataDxfId="56" totalsRowDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="SEQ" dataDxfId="55" totalsRowDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Q1" dataDxfId="54" totalsRowDxfId="5"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Q2" dataDxfId="53" totalsRowDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Q3" dataDxfId="52" totalsRowDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Q4" dataDxfId="51" totalsRowDxfId="2"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Q5" dataDxfId="50" totalsRowDxfId="1"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Q6" dataDxfId="49" totalsRowDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Final" dataDxfId="61" totalsRowDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1" dataDxfId="60" totalsRowDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="2" dataDxfId="59" totalsRowDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="3" dataDxfId="58" totalsRowDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="4" dataDxfId="57" totalsRowDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="5" dataDxfId="56" totalsRowDxfId="8"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="6" dataDxfId="55" totalsRowDxfId="7"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="SEQ" dataDxfId="54" totalsRowDxfId="6"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Q1" dataDxfId="53" totalsRowDxfId="5"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Q2" dataDxfId="52" totalsRowDxfId="4"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Q3" dataDxfId="51" totalsRowDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Q4" dataDxfId="50" totalsRowDxfId="2"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Q5" dataDxfId="49" totalsRowDxfId="1"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Q6" dataDxfId="48" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="48" dataDxfId="47" totalsRowDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="47" dataDxfId="46" totalsRowDxfId="45">
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="40"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="39"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="38"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="37"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="35"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="34"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="33"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="32"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="31"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="30"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="37"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="35"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="34"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="33"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="32"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="31"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="30"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="29"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3962,7 +3962,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:B19">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Model"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3973,7 +3973,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Standard"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Concept"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3985,7 +3985,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="#"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Framework"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Specifications"/>
-    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="26">
+    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="25">
       <calculatedColumnFormula>_xlfn.CONCAT(Table3[[#This Row],['#]],": ",Table3[[#This Row],[Framework]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6520,7 +6520,9 @@
       <c r="P29" s="1">
         <v>2</v>
       </c>
-      <c r="Q29" s="28"/>
+      <c r="Q29" s="28">
+        <v>2</v>
+      </c>
       <c r="R29" s="1">
         <f>IF(K29=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -6597,7 +6599,9 @@
         <v>1</v>
       </c>
       <c r="P30" s="1"/>
-      <c r="Q30" s="28"/>
+      <c r="Q30" s="28">
+        <v>2</v>
+      </c>
       <c r="R30" s="1">
         <f>IF(K30=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -6676,7 +6680,9 @@
       <c r="P31" s="1">
         <v>2</v>
       </c>
-      <c r="Q31" s="28"/>
+      <c r="Q31" s="28">
+        <v>0</v>
+      </c>
       <c r="R31" s="1">
         <f>IF(K31=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -6834,7 +6840,9 @@
       <c r="P33" s="1">
         <v>3</v>
       </c>
-      <c r="Q33" s="28"/>
+      <c r="Q33" s="28">
+        <v>2</v>
+      </c>
       <c r="R33" s="1">
         <f>IF(K33=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -6913,7 +6921,9 @@
       <c r="P34" s="1">
         <v>1</v>
       </c>
-      <c r="Q34" s="28"/>
+      <c r="Q34" s="28">
+        <v>0</v>
+      </c>
       <c r="R34" s="1">
         <f>IF(K34=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -6992,7 +7002,9 @@
       <c r="P35" s="1">
         <v>2</v>
       </c>
-      <c r="Q35" s="28"/>
+      <c r="Q35" s="28">
+        <v>0</v>
+      </c>
       <c r="R35" s="1">
         <f>IF(K35=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -7071,7 +7083,9 @@
       <c r="P36" s="1">
         <v>2</v>
       </c>
-      <c r="Q36" s="28"/>
+      <c r="Q36" s="28">
+        <v>4</v>
+      </c>
       <c r="R36" s="1">
         <f>IF(K36=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -7229,7 +7243,9 @@
       <c r="P38" s="1">
         <v>2</v>
       </c>
-      <c r="Q38" s="28"/>
+      <c r="Q38" s="28">
+        <v>3</v>
+      </c>
       <c r="R38" s="1">
         <f>IF(K38=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -7308,7 +7324,9 @@
       <c r="P39" s="1">
         <v>2</v>
       </c>
-      <c r="Q39" s="28"/>
+      <c r="Q39" s="28">
+        <v>1</v>
+      </c>
       <c r="R39" s="1">
         <f>IF(K39=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -7387,7 +7405,9 @@
       <c r="P40" s="1">
         <v>1</v>
       </c>
-      <c r="Q40" s="28"/>
+      <c r="Q40" s="28">
+        <v>2</v>
+      </c>
       <c r="R40" s="1">
         <f>IF(K40=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -7466,7 +7486,9 @@
       <c r="P41" s="1">
         <v>2</v>
       </c>
-      <c r="Q41" s="28"/>
+      <c r="Q41" s="28">
+        <v>3</v>
+      </c>
       <c r="R41" s="1">
         <f>IF(K41=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -7545,7 +7567,9 @@
       <c r="P42" s="1">
         <v>2</v>
       </c>
-      <c r="Q42" s="28"/>
+      <c r="Q42" s="28">
+        <v>0</v>
+      </c>
       <c r="R42" s="1">
         <f>IF(K42=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -7624,7 +7648,9 @@
       <c r="P43" s="1">
         <v>2</v>
       </c>
-      <c r="Q43" s="28"/>
+      <c r="Q43" s="28">
+        <v>2</v>
+      </c>
       <c r="R43" s="1">
         <f>IF(K43=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -7703,7 +7729,9 @@
       <c r="P44" s="1">
         <v>4</v>
       </c>
-      <c r="Q44" s="28"/>
+      <c r="Q44" s="28">
+        <v>4</v>
+      </c>
       <c r="R44" s="1">
         <f>IF(K44=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>0</v>
@@ -7853,7 +7881,9 @@
       <c r="P46" s="1">
         <v>2</v>
       </c>
-      <c r="Q46" s="28"/>
+      <c r="Q46" s="28">
+        <v>1</v>
+      </c>
       <c r="R46" s="1">
         <f>IF(K46=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
         <v>1</v>
@@ -13074,7 +13104,7 @@
   </sheetData>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="K2:P120">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="24" priority="1">
       <formula>R2=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13513,7 +13543,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:I8">
-    <cfRule type="expression" dxfId="24" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>"Option_"&amp;$E2=F$1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Regenerated with new colors
</commit_message>
<xml_diff>
--- a/US/October CMA/US October CMA Data.xlsx
+++ b/US/October CMA/US October CMA Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/coledushin/Documents/GWHS/US/October CMA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1809095C-331E-FA4C-B427-575B19AFBA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{725D73EA-3A62-DD4A-B822-CEB06083DCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="889">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="891">
   <si>
     <t>Model</t>
   </si>
@@ -2706,6 +2706,12 @@
   </si>
   <si>
     <t>OYI76487</t>
+  </si>
+  <si>
+    <t>QVB46757</t>
+  </si>
+  <si>
+    <t>MJB56814</t>
   </si>
 </sst>
 </file>
@@ -2843,7 +2849,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -2878,43 +2884,6 @@
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="FFD8E0E8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FFD8E0E8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FFD8E0E8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F4A58"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FFD8E0E8"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -2985,7 +2954,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3056,31 +3025,79 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3090,19 +3107,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -3110,61 +3115,25 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -3172,7 +3141,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -3180,19 +3149,19 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -3200,7 +3169,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -3208,41 +3177,23 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="13" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3252,7 +3203,17 @@
     <cellStyle name="Normal 4" xfId="3" xr:uid="{D605B4E0-7730-4D43-A011-6A0EF9292E1A}"/>
     <cellStyle name="Percent 2" xfId="4" xr:uid="{E6DE421D-B06A-DB4D-BCE7-D696BB42B3F4}"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="33">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -3509,10 +3470,10 @@
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Light and Airy" count="4" xr9:uid="{9857ACD9-B079-C44A-A030-69F7726DB419}">
-      <tableStyleElement type="wholeTable" dxfId="31"/>
-      <tableStyleElement type="headerRow" dxfId="30"/>
-      <tableStyleElement type="totalRow" dxfId="29"/>
-      <tableStyleElement type="firstRowStripe" dxfId="28"/>
+      <tableStyleElement type="wholeTable" dxfId="32"/>
+      <tableStyleElement type="headerRow" dxfId="31"/>
+      <tableStyleElement type="totalRow" dxfId="30"/>
+      <tableStyleElement type="firstRowStripe" dxfId="29"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -3550,10 +3511,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C04EAAE0-8575-4C4D-8F7C-680B0F8FE844}" name="Table4" displayName="Table4" ref="A1:U141" totalsRowShown="0" headerRowDxfId="27" tableBorderDxfId="26">
-  <autoFilter ref="A1:U141" xr:uid="{C04EAAE0-8575-4C4D-8F7C-680B0F8FE844}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C04EAAE0-8575-4C4D-8F7C-680B0F8FE844}" name="Table4" displayName="Table4" ref="A1:U142" totalsRowShown="0" headerRowDxfId="28" tableBorderDxfId="27">
+  <autoFilter ref="A1:U142" xr:uid="{C04EAAE0-8575-4C4D-8F7C-680B0F8FE844}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{C8800E54-CA52-2044-A16A-FF3249E700E8}" name="Key" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{C8800E54-CA52-2044-A16A-FF3249E700E8}" name="Key" dataDxfId="26"/>
     <tableColumn id="5" xr3:uid="{1508E423-CBEF-6F4B-9DCF-7D205ACAAA4A}" name="Class"/>
     <tableColumn id="6" xr3:uid="{AACC7F38-4163-B84F-88F9-448EEF83552D}" name="Period"/>
     <tableColumn id="7" xr3:uid="{1050C21B-C0F8-E841-8048-E0D87CBF2D06}" name="Grade"/>
@@ -3580,25 +3541,25 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Questions" displayName="Questions" ref="A1:Q8" headerRowDxfId="25" dataDxfId="24" totalsRowDxfId="23">
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Part" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stimulus" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Question" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Key" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Option_1" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Option_2" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Option_3" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Option_4" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="Stimulus_type" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Source_type" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Task_model" dataDxfId="11"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0100-00000D000000}" name="Skill_standard" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0100-00000E000000}" name="Need_OI?" dataDxfId="9"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0100-00000F000000}" name="Content_standard" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0100-000010000000}" name="Pct_Correct" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0100-000011000000}" name="Point_Biserial" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3608,7 +3569,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:B19">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Model"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Detail" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3619,7 +3580,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Standard"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Concept"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Specification" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="Light and Airy" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3631,7 +3592,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="#"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Framework"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Specifications"/>
-    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="2">
+    <tableColumn id="4" xr3:uid="{B9670A8F-2834-6A44-B0B5-70CE5D45B362}" name="Concatenated" dataDxfId="3">
       <calculatedColumnFormula>_xlfn.CONCAT(Table3[[#This Row],['#]],": ",Table3[[#This Row],[Framework]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3862,7 +3823,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W141"/>
+  <dimension ref="A1:W142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="21" customHeight="1" outlineLevelCol="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="10.5" style="20" bestFit="1" customWidth="1"/>
@@ -3879,7 +3840,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="18" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="64" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="26" t="s">
@@ -13494,43 +13455,155 @@
       </c>
     </row>
     <row r="141" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A141" s="71"/>
-      <c r="B141" s="64"/>
-      <c r="C141" s="65"/>
-      <c r="D141" s="65"/>
-      <c r="E141" s="66"/>
-      <c r="F141" s="67"/>
-      <c r="G141" s="68">
-        <f>AVERAGE(Scores!$G$2:$G$140)</f>
-        <v>3.5323741007194243</v>
-      </c>
-      <c r="H141" s="64"/>
-      <c r="I141" s="69"/>
-      <c r="J141" s="65"/>
-      <c r="K141" s="65"/>
-      <c r="L141" s="65"/>
-      <c r="M141" s="65"/>
-      <c r="N141" s="65"/>
-      <c r="O141" s="69"/>
-      <c r="P141" s="69"/>
-      <c r="Q141" s="65"/>
-      <c r="R141" s="65"/>
-      <c r="S141" s="65"/>
-      <c r="T141" s="65"/>
-      <c r="U141" s="65"/>
+      <c r="A141" s="20" t="s">
+        <v>889</v>
+      </c>
+      <c r="B141" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C141" s="20">
+        <v>4</v>
+      </c>
+      <c r="D141" s="20">
+        <v>9</v>
+      </c>
+      <c r="E141" s="23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F141" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G141" s="20">
+        <v>3</v>
+      </c>
+      <c r="H141" s="65"/>
+      <c r="I141" s="20">
+        <v>2</v>
+      </c>
+      <c r="J141" s="20">
+        <v>1</v>
+      </c>
+      <c r="K141" s="20">
+        <v>3</v>
+      </c>
+      <c r="L141" s="20">
+        <v>3</v>
+      </c>
+      <c r="M141" s="20">
+        <v>3</v>
+      </c>
+      <c r="N141" s="20">
+        <v>2</v>
+      </c>
+      <c r="O141" s="22">
+        <v>1</v>
+      </c>
+      <c r="P141" s="46">
+        <f>IF(I141=VLOOKUP(VALUE(I$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q141" s="43">
+        <f>IF(J141=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R141" s="43">
+        <f>IF(K141=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S141" s="43">
+        <f>IF(L141=VLOOKUP(VALUE(L$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T141" s="43">
+        <f>IF(M141=VLOOKUP(VALUE(M$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U141" s="43">
+        <f>IF(N141=VLOOKUP(VALUE(N$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A142" s="20" t="s">
+        <v>890</v>
+      </c>
+      <c r="B142" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C142" s="20">
+        <v>4</v>
+      </c>
+      <c r="D142" s="20">
+        <v>9</v>
+      </c>
+      <c r="E142" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="F142" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G142" s="20">
+        <v>1</v>
+      </c>
+      <c r="H142" s="65"/>
+      <c r="I142" s="20">
+        <v>2</v>
+      </c>
+      <c r="J142" s="20">
+        <v>4</v>
+      </c>
+      <c r="K142" s="20">
+        <v>3</v>
+      </c>
+      <c r="L142" s="20">
+        <v>1</v>
+      </c>
+      <c r="M142" s="20">
+        <v>3</v>
+      </c>
+      <c r="N142" s="20">
+        <v>3</v>
+      </c>
+      <c r="O142" s="22">
+        <v>1</v>
+      </c>
+      <c r="P142" s="46">
+        <f>IF(I142=VLOOKUP(VALUE(I$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q142" s="43">
+        <f>IF(J142=VLOOKUP(VALUE(J$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R142" s="43">
+        <f>IF(K142=VLOOKUP(VALUE(K$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S142" s="43">
+        <f>IF(L142=VLOOKUP(VALUE(L$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="T142" s="43">
+        <f>IF(M142=VLOOKUP(VALUE(M$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U142" s="43">
+        <f>IF(N142=VLOOKUP(VALUE(N$1),Questions[#All],5,FALSE),1,0)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="12" type="noConversion"/>
-  <conditionalFormatting sqref="I2:N140">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="I2:N142">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
       <formula>P2=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="B2:B140" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B142" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Bermejo,Dushin,Klein / Cooper,Kovelsky"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="H2:H140" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="H2:H142" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>AND(ISNUMBER(H2),(NOT(OR(NOT(ISERROR(DATEVALUE(H2))), AND(ISNUMBER(H2), LEFT(CELL("format", H2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>
@@ -13663,8 +13736,8 @@
         <v>743</v>
       </c>
       <c r="P2" s="15">
-        <f t="array" ref="P2">AVERAGE(INDEX(Scores!$B$2:$U$140,0,MATCH("Q"&amp;$A2,Scores!$B$1:$U$1,0)))</f>
-        <v>0.52517985611510787</v>
+        <f t="array" ref="P2">AVERAGE(INDEX(Scores!$B$2:$U$142,0,MATCH("Q"&amp;$A2,Scores!$B$1:$U$1,0)))</f>
+        <v>0.51773049645390068</v>
       </c>
       <c r="Q2" s="13"/>
     </row>
@@ -13715,8 +13788,8 @@
         <v>743</v>
       </c>
       <c r="P3" s="15">
-        <f t="array" ref="P3">AVERAGE(INDEX(Scores!$B$2:$U$140,0,MATCH("Q"&amp;$A3,Scores!$B$1:$U$1,0)))</f>
-        <v>0.49640287769784175</v>
+        <f t="array" ref="P3">AVERAGE(INDEX(Scores!$B$2:$U$142,0,MATCH("Q"&amp;$A3,Scores!$B$1:$U$1,0)))</f>
+        <v>0.49645390070921985</v>
       </c>
       <c r="Q3" s="13"/>
     </row>
@@ -13767,8 +13840,8 @@
         <v>745</v>
       </c>
       <c r="P4" s="15">
-        <f t="array" ref="P4">AVERAGE(INDEX(Scores!$B$2:$U$140,0,MATCH("Q"&amp;$A4,Scores!$B$1:$U$1,0)))</f>
-        <v>0.79856115107913672</v>
+        <f t="array" ref="P4">AVERAGE(INDEX(Scores!$B$2:$U$142,0,MATCH("Q"&amp;$A4,Scores!$B$1:$U$1,0)))</f>
+        <v>0.8014184397163121</v>
       </c>
       <c r="Q4" s="13"/>
     </row>
@@ -13819,8 +13892,8 @@
         <v>745</v>
       </c>
       <c r="P5" s="15">
-        <f t="array" ref="P5">AVERAGE(INDEX(Scores!$B$2:$U$140,0,MATCH("Q"&amp;$A5,Scores!$B$1:$U$1,0)))</f>
-        <v>0.73381294964028776</v>
+        <f t="array" ref="P5">AVERAGE(INDEX(Scores!$B$2:$U$142,0,MATCH("Q"&amp;$A5,Scores!$B$1:$U$1,0)))</f>
+        <v>0.72340425531914898</v>
       </c>
       <c r="Q5" s="13"/>
     </row>
@@ -13871,8 +13944,8 @@
         <v>746</v>
       </c>
       <c r="P6" s="15">
-        <f t="array" ref="P6">AVERAGE(INDEX(Scores!$B$2:$U$140,0,MATCH("Q"&amp;$A6,Scores!$B$1:$U$1,0)))</f>
-        <v>0.34532374100719426</v>
+        <f t="array" ref="P6">AVERAGE(INDEX(Scores!$B$2:$U$142,0,MATCH("Q"&amp;$A6,Scores!$B$1:$U$1,0)))</f>
+        <v>0.3546099290780142</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
@@ -13923,8 +13996,8 @@
         <v>746</v>
       </c>
       <c r="P7" s="15">
-        <f t="array" ref="P7">AVERAGE(INDEX(Scores!$B$2:$U$140,0,MATCH("Q"&amp;$A7,Scores!$B$1:$U$1,0)))</f>
-        <v>0.67625899280575541</v>
+        <f t="array" ref="P7">AVERAGE(INDEX(Scores!$B$2:$U$142,0,MATCH("Q"&amp;$A7,Scores!$B$1:$U$1,0)))</f>
+        <v>0.67375886524822692</v>
       </c>
       <c r="Q7" s="13"/>
     </row>
@@ -13961,7 +14034,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:I8">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>"Option_"&amp;$E2=F$1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>